<commit_message>
Remove decision on households
</commit_message>
<xml_diff>
--- a/model/Inputs/inputs.xlsx
+++ b/model/Inputs/inputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailaub-my.sharepoint.com/personal/mo10_aub_edu_lb/Documents/3-Research/Elsa/Model 1/Github/Model-1/model/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="229" documentId="6_{7DA8CDEE-914B-4384-BE83-347F050180D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A30ECDE8-D5BD-43E1-9AE8-19ED56EE62A2}"/>
+  <xr:revisionPtr revIDLastSave="233" documentId="6_{7DA8CDEE-914B-4384-BE83-347F050180D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9E27A5E-4AB9-4FF6-9338-6D51785C5180}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="parameters" sheetId="1" r:id="rId1"/>
@@ -320,6 +320,10 @@
     <mc:Fallback/>
   </mc:AlternateContent>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1617,153 +1621,153 @@
         <v>21</v>
       </c>
       <c r="B2">
-        <v>0.2623351352601862</v>
+        <v>0.50966710862198827</v>
       </c>
       <c r="C2">
-        <v>0.17062120330461161</v>
+        <v>0.5378994808540265</v>
       </c>
       <c r="D2">
-        <v>0.2092049542430571</v>
+        <v>0.53090703423607699</v>
       </c>
       <c r="E2">
-        <v>0.28747276823387014</v>
+        <v>0.53124301708715971</v>
       </c>
       <c r="F2">
-        <v>0.36604134920128423</v>
+        <v>0.52153379679324718</v>
       </c>
       <c r="G2">
-        <v>0.41222889257948481</v>
+        <v>0.49426688993448104</v>
       </c>
       <c r="H2">
-        <v>0.36872864366248936</v>
+        <v>0.42588406065382994</v>
       </c>
       <c r="I2">
-        <v>0.34093467439274378</v>
+        <v>0.38927000806723039</v>
       </c>
       <c r="J2">
-        <v>0.29284143627333531</v>
+        <v>0.32784201041527922</v>
       </c>
       <c r="K2">
-        <v>0.37229578188674872</v>
+        <v>0.39403786103913829</v>
       </c>
       <c r="L2">
-        <v>0.40984403001373088</v>
+        <v>0.42387390011083459</v>
       </c>
       <c r="M2">
-        <v>0.40508530223820943</v>
+        <v>0.41429178637998687</v>
       </c>
       <c r="N2">
-        <v>0.40344423654076739</v>
+        <v>0.41261342373487581</v>
       </c>
       <c r="O2">
-        <v>0.38165770479616301</v>
+        <v>0.41384570399583948</v>
       </c>
       <c r="P2">
-        <v>0.37891608840766111</v>
+        <v>0.41587988599549158</v>
       </c>
       <c r="Q2">
-        <v>0.37389510552131089</v>
+        <v>0.39982959439825999</v>
       </c>
       <c r="R2">
-        <v>0.38774062129651121</v>
+        <v>0.38773501471725841</v>
       </c>
       <c r="S2">
         <v>0.3186474998936335</v>
       </c>
       <c r="T2">
-        <v>0.24380642028312829</v>
+        <v>0.25054140426885008</v>
       </c>
       <c r="U2">
-        <v>0.25395866140635881</v>
+        <v>0.27056497061016371</v>
       </c>
       <c r="V2">
-        <v>0.29588047973401582</v>
+        <v>0.36064017729795278</v>
       </c>
       <c r="W2">
-        <v>0.30127927607913685</v>
+        <v>0.39697265447803048</v>
       </c>
       <c r="X2">
-        <v>0.32115797413359637</v>
+        <v>0.42768970618440738</v>
       </c>
       <c r="Y2">
-        <v>0.36269677918310511</v>
+        <v>0.4793303803666743</v>
       </c>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="4">
-        <v>0.15382816766586732</v>
-      </c>
-      <c r="C3" s="4">
-        <v>0.13016580775379691</v>
-      </c>
-      <c r="D3" s="4">
-        <v>0.110470854616307</v>
-      </c>
-      <c r="E3" s="4">
-        <v>9.7743641686650659E-2</v>
-      </c>
-      <c r="F3" s="4">
-        <v>4.7205897881694631E-2</v>
-      </c>
-      <c r="G3" s="4">
-        <v>1.289322322142287E-2</v>
-      </c>
-      <c r="H3" s="4">
-        <v>3.3261776673661064E-2</v>
-      </c>
-      <c r="I3" s="4">
-        <v>0.11926557690297759</v>
-      </c>
-      <c r="J3" s="4">
-        <v>0.1072343263734013</v>
-      </c>
-      <c r="K3" s="4">
-        <v>7.2847478437250215E-2</v>
-      </c>
-      <c r="L3" s="4">
-        <v>0.1064278170953237</v>
-      </c>
-      <c r="M3" s="4">
-        <v>5.0854727103317371E-2</v>
-      </c>
-      <c r="N3" s="4">
-        <v>7.3324414341027169E-2</v>
-      </c>
-      <c r="O3" s="4">
-        <v>0.1443651041966427</v>
-      </c>
-      <c r="P3" s="4">
-        <v>9.895206895983219E-2</v>
-      </c>
-      <c r="Q3" s="4">
-        <v>3.5798383593125475E-2</v>
-      </c>
-      <c r="R3" s="4">
-        <v>6.3494702238209397E-2</v>
-      </c>
-      <c r="S3" s="4">
-        <v>1.786535421662672E-2</v>
-      </c>
-      <c r="T3" s="4">
-        <v>2.0976981115107929E-2</v>
-      </c>
-      <c r="U3" s="4">
-        <v>4.7162871828037585E-2</v>
-      </c>
-      <c r="V3" s="4">
-        <v>2.771126862509992E-2</v>
-      </c>
-      <c r="W3" s="4">
-        <v>3.5392782224220605E-2</v>
-      </c>
-      <c r="X3" s="4">
-        <v>4.6282933453237439E-2</v>
-      </c>
-      <c r="Y3" s="4">
-        <v>0.11903915947242209</v>
+      <c r="B3">
+        <v>0.21451117157625252</v>
+      </c>
+      <c r="C3">
+        <v>0.201505708253541</v>
+      </c>
+      <c r="D3">
+        <v>0.18470652041524671</v>
+      </c>
+      <c r="E3">
+        <v>0.18225432239922348</v>
+      </c>
+      <c r="F3">
+        <v>0.1554154603117506</v>
+      </c>
+      <c r="G3">
+        <v>0.1117803120003997</v>
+      </c>
+      <c r="H3">
+        <v>9.0519316070893294E-2</v>
+      </c>
+      <c r="I3">
+        <v>3.6473810596522891E-3</v>
+      </c>
+      <c r="J3">
+        <v>6.4906675934941482E-3</v>
+      </c>
+      <c r="K3">
+        <v>1.3591447442735459E-2</v>
+      </c>
+      <c r="L3">
+        <v>2.2364190957251128E-2</v>
+      </c>
+      <c r="M3">
+        <v>3.1440585337638952E-2</v>
+      </c>
+      <c r="N3">
+        <v>8.5988232895579907E-3</v>
+      </c>
+      <c r="O3">
+        <v>7.2333525303942922E-2</v>
+      </c>
+      <c r="P3">
+        <v>1.866558683208901E-2</v>
+      </c>
+      <c r="Q3">
+        <v>6.6216998886605011E-2</v>
+      </c>
+      <c r="R3">
+        <v>2.0066803971457031E-2</v>
+      </c>
+      <c r="S3">
+        <v>8.3773723157837349E-2</v>
+      </c>
+      <c r="T3">
+        <v>0.1144162737037261</v>
+      </c>
+      <c r="U3">
+        <v>0.16986397859008559</v>
+      </c>
+      <c r="V3">
+        <v>0.20655493073070949</v>
+      </c>
+      <c r="W3">
+        <v>0.22152122671408322</v>
+      </c>
+      <c r="X3">
+        <v>0.20763276923213911</v>
+      </c>
+      <c r="Y3">
+        <v>0.2348585481078552</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.35">
@@ -1771,76 +1775,76 @@
         <v>23</v>
       </c>
       <c r="B4">
-        <v>6.6497939365097805E-2</v>
+        <v>8.005597698503418E-2</v>
       </c>
       <c r="C4">
-        <v>6.0829684742988738E-3</v>
+        <v>7.7211791688954104E-2</v>
       </c>
       <c r="D4">
-        <v>3.6389563487457531E-4</v>
+        <v>5.5918791628873997E-2</v>
       </c>
       <c r="E4">
-        <v>7.0017249552892222E-2</v>
+        <v>1.0642524735926339E-2</v>
       </c>
       <c r="F4">
-        <v>3.6004447702206885E-2</v>
+        <v>3.9543081047258954E-2</v>
       </c>
       <c r="G4">
-        <v>2.9453637187024581E-2</v>
+        <v>8.6450810668165581E-2</v>
       </c>
       <c r="H4">
-        <v>4.8533218738373358E-2</v>
+        <v>0.14607880221876421</v>
       </c>
       <c r="I4">
-        <v>9.2245401997986864E-2</v>
+        <v>0.17308492085455379</v>
       </c>
       <c r="J4">
-        <v>9.9277797118296138E-2</v>
+        <v>0.19612612231534801</v>
       </c>
       <c r="K4">
-        <v>0.12859123949826309</v>
+        <v>0.2120407695560845</v>
       </c>
       <c r="L4">
-        <v>0.120883134786871</v>
+        <v>0.24076334244371791</v>
       </c>
       <c r="M4">
-        <v>0.19811139155647978</v>
+        <v>0.2515475077754965</v>
       </c>
       <c r="N4">
-        <v>0.19275881941213541</v>
+        <v>0.22804079980856531</v>
       </c>
       <c r="O4">
-        <v>0.16332418525123069</v>
+        <v>0.24612502923546858</v>
       </c>
       <c r="P4">
-        <v>0.13845818331804599</v>
+        <v>0.24122140464981048</v>
       </c>
       <c r="Q4">
-        <v>0.17321570969695821</v>
+        <v>0.25383203669113041</v>
       </c>
       <c r="R4">
-        <v>0.2311011628004816</v>
+        <v>0.27166616365594148</v>
       </c>
       <c r="S4">
-        <v>0.14675733461978502</v>
+        <v>0.2293876512998364</v>
       </c>
       <c r="T4">
-        <v>9.9394006227721363E-2</v>
+        <v>0.1350092828668254</v>
       </c>
       <c r="U4">
-        <v>0.17673245022317011</v>
+        <v>0.20668343356313848</v>
       </c>
       <c r="V4">
-        <v>1.839866574382585E-2</v>
+        <v>0.1208918472888901</v>
       </c>
       <c r="W4">
-        <v>0.1238525089555544</v>
+        <v>0.2060606107426603</v>
       </c>
       <c r="X4">
-        <v>1.250104770477016E-2</v>
+        <v>0.1022593244130014</v>
       </c>
       <c r="Y4">
-        <v>2.3547867286155183E-2</v>
+        <v>0.11364610358988639</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.35">
@@ -2345,6 +2349,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D835CF4C7D56B243BA013D4D2E10914B" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2e645ef68b9493f2ee8bae9e534bc24f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="6d4e152b-60f6-4719-8921-68b5b8011cde" xmlns:ns4="28683373-984a-4841-9f0e-018f3f7bab1f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a06da6e71fc3d3bdf7cbe176c2a8afa1" ns3:_="" ns4:_="">
     <xsd:import namespace="6d4e152b-60f6-4719-8921-68b5b8011cde"/>
@@ -2597,15 +2610,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2615,6 +2619,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DCE34160-36D4-4F46-97A9-A281FB44CDD4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCE4FBA5-6C26-4B97-9218-92B658F853C9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2629,14 +2641,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DCE34160-36D4-4F46-97A9-A281FB44CDD4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Run outputs and a plots
</commit_message>
<xml_diff>
--- a/model/Inputs/inputs.xlsx
+++ b/model/Inputs/inputs.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Elsa\OneDrive - American University of Beirut\Masters\Research\Elsa\Model 1\Github\Model-1\model\Inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailaub-my.sharepoint.com/personal/mo10_aub_edu_lb/Documents/3-Research/Elsa/Model 1/Github/Model-1/model/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAD2F7EF-0845-4A2E-9423-0E1C0E08F108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{AAD2F7EF-0845-4A2E-9423-0E1C0E08F108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{353AE6E4-AFA5-4B68-AD1B-B2C80ADE73C4}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1706,10 +1706,10 @@
         <v>0.30451730640166025</v>
       </c>
       <c r="F3">
-        <v>9.6890092592592555E-2</v>
+        <v>0.28329803098345968</v>
       </c>
       <c r="G3">
-        <v>5.3708466145833411E-2</v>
+        <v>0.26207875556525934</v>
       </c>
       <c r="H3">
         <v>0.2408594801470588</v>
@@ -1780,7 +1780,7 @@
         <v>0.21363559324698039</v>
       </c>
       <c r="E4">
-        <v>0.1516221565352886</v>
+        <v>0.20448834535510552</v>
       </c>
       <c r="F4">
         <v>0.19534109746323072</v>
@@ -2345,15 +2345,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_activity xmlns="6d4e152b-60f6-4719-8921-68b5b8011cde" xsi:nil="true"/>
@@ -2361,7 +2352,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D835CF4C7D56B243BA013D4D2E10914B" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2e645ef68b9493f2ee8bae9e534bc24f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="6d4e152b-60f6-4719-8921-68b5b8011cde" xmlns:ns4="28683373-984a-4841-9f0e-018f3f7bab1f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a06da6e71fc3d3bdf7cbe176c2a8afa1" ns3:_="" ns4:_="">
     <xsd:import namespace="6d4e152b-60f6-4719-8921-68b5b8011cde"/>
@@ -2614,15 +2605,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DCE34160-36D4-4F46-97A9-A281FB44CDD4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E95B8A76-94F3-412F-9855-4B93BB4C4C10}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2639,7 +2631,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCE4FBA5-6C26-4B97-9218-92B658F853C9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2656,4 +2648,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DCE34160-36D4-4F46-97A9-A281FB44CDD4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>